<commit_message>
Verifica settimanale: 91 upgrade doppio controllo, stato/log aggiornati
Completa il run di verifica settimanale: applica i 91 upgrade a
"VERIFICATA AI - doppio controllo" dai 9 agenti paralleli di ricerca
web (175/243 candidati raggiunti su 243 prima dell'esaurimento quota
WebSearch condiviso), aggiorna weekly_verify_state.json (last_run_at,
421 file processati) e weekly_verify_log.md con il riepilogo del run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KaU1epvovxEPcBHjxGKYw
</commit_message>
<xml_diff>
--- a/output/2026-10-05_15_Malesia_Terengganu_Metalworking_Lavorazioni_Metalliche.xlsx
+++ b/output/2026-10-05_15_Malesia_Terengganu_Metalworking_Lavorazioni_Metalliche.xlsx
@@ -520,7 +520,6 @@
           <t>WTC Hardware &amp; Industrial Supply Sdn. Bhd.</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Cukai, Kemaman, Terengganu</t>
@@ -536,7 +535,6 @@
           <t>019-9863098</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Attiva dal 1996. Indirizzo: K7332, Jalan Jakar, Cukai, 24000 Kemaman. Fonte: newpages.com.my, glbosun.com.my, dongchengmalaysia.com.</t>
@@ -574,7 +572,6 @@
           <t>+60 17-891 7113 (WhatsApp)</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Indirizzo: Lot 3577 Jalan Awana 1, Bukit Kuang, Kemaman. Verificato tramite sito ufficiale.</t>
@@ -634,7 +631,6 @@
           <t>TLH Hardware &amp; Machinery Sdn. Bhd.</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Paka, Dungun, Terengganu</t>
@@ -650,7 +646,6 @@
           <t>09-827 2364</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>Esistenza confermata da piu' directory (EMIS, Yelp, contact.page). ATTENZIONE: registrato anche presso CIDB come contractor edile G5 (Other Foundation, Structure and Building Exterior Contractors) - verificare se l'attivita' prevalente e' distribuzione hardware o edilizia.</t>
@@ -668,7 +663,6 @@
           <t>LK Hardware &amp; Machinery Trading Sdn. Bhd.</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Paka, Dungun, Terengganu</t>
@@ -684,7 +678,6 @@
           <t>+6098281633</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Costituita nel 1993. Indirizzo: Lot 2434, Jalan Besar, Paka, 23100 Terengganu. Fonte: EMIS, businesslist.my.</t>
@@ -702,7 +695,6 @@
           <t>JJ Machinery &amp; Hardware Sdn. Bhd.</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Kuala Terengganu</t>
@@ -718,7 +710,6 @@
           <t>09-626 2333</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Indirizzo: 40-B &amp; C, Jalan Hiliran, Kuala Terengganu. Fonte: Yelp, panpages.my.</t>
@@ -736,7 +727,6 @@
           <t>Yong Seng Machinery Supply &amp; Trading</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Kuala Terengganu</t>
@@ -752,7 +742,6 @@
           <t>09-622 2558</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Indirizzo: No. 83, 83A &amp; 83B, Jalan Losong Feri, Kuala Terengganu. Esistenza confermata (mypages.my, contact.page); numero telefono fornito in lista originale non riverificato in modo indipendente al 100% (fonti mostrano prefisso coerente ma oscurato).</t>
@@ -770,7 +759,6 @@
           <t>Ciri Bina Machinery &amp; Hardware Sdn Bhd</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Kuala Terengganu</t>
@@ -781,8 +769,6 @@
           <t>Macchinari e hardware (wholesale trade)</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>Esistenza confermata tramite directory Dun &amp; Bradstreet, categoria Machinery, Equipment and Supplies Merchant Wholesalers. Indirizzo e contatti diretti non reperiti.</t>
@@ -800,7 +786,6 @@
           <t>Aimgas Sdn. Bhd.</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>Kuala Terengganu</t>
@@ -811,8 +796,6 @@
           <t>Attrezzature e forniture per saldatura, hardware</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Esistenza confermata tramite directory (malaysia.contact.page). Indirizzo: Lot 1742, Jalan Sultan Mohamad, Kuala Terengganu. Contatti diretti non reperiti.</t>
@@ -862,7 +845,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (12/10/2026)</t>
         </is>
       </c>
     </row>
@@ -872,7 +855,6 @@
           <t>Teozon Centre</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Kubang Parit, Kuala Terengganu</t>
@@ -888,7 +870,6 @@
           <t>019-7799802</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>Negozio di ferramenta confermato (Foursquare). Indirizzo: 197-A, Jalan Kelantan Lama, Kg Durian Burung, Kubang Parit, 20050 Kuala Terengganu.</t>

</xml_diff>